<commit_message>
add requisites module and restore admin design
</commit_message>
<xml_diff>
--- a/p-word list.xlsx
+++ b/p-word list.xlsx
@@ -1,22 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\work-system\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0B1CC17-BCE0-475F-A5E0-BF1B67BD4107}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="384" yWindow="132" windowWidth="22020" windowHeight="8760"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
     <sheet name="Лист2" sheetId="2" r:id="rId2"/>
     <sheet name="Лист3" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="145621"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="253">
   <si>
     <t>Байбулатова Татьяна Николаевна</t>
   </si>
@@ -769,12 +789,18 @@
   </si>
   <si>
     <t>employee_name</t>
+  </si>
+  <si>
+    <t>Карпова Екатерина Николаевна</t>
+  </si>
+  <si>
+    <t>Pass201</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -817,8 +843,29 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CA9F819E-E91C-4626-AA0D-9A1C84CA540B}" name="Таблица1" displayName="Таблица1" ref="A1:C126" totalsRowShown="0">
+  <autoFilter ref="A1:C126" xr:uid="{CA9F819E-E91C-4626-AA0D-9A1C84CA540B}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="Абдикаоров Асадбек Баодирович"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{677094AA-556F-4B74-808C-808F917AAAED}" name="phone"/>
+    <tableColumn id="2" xr3:uid="{C7201A3C-E2D4-4488-A729-24D9733602F8}" name="employee_name"/>
+    <tableColumn id="3" xr3:uid="{0068CC08-34CF-45B9-9A91-138CD5E59319}" name="password"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -864,7 +911,7 @@
     </a:clrScheme>
     <a:fontScheme name="Стандартная">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -897,9 +944,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -932,6 +996,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Стандартная">
@@ -1107,16 +1188,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C125"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C126"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="38.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -1127,7 +1208,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>79216379168</v>
       </c>
@@ -1138,7 +1219,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>79215854629</v>
       </c>
@@ -1149,7 +1230,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>79921952699</v>
       </c>
@@ -1160,7 +1241,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>79052112426</v>
       </c>
@@ -1171,7 +1252,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>79500346601</v>
       </c>
@@ -1182,7 +1263,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>79112309976</v>
       </c>
@@ -1193,7 +1274,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>79817651223</v>
       </c>
@@ -1204,7 +1285,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>79110865055</v>
       </c>
@@ -1215,7 +1296,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>79522081319</v>
       </c>
@@ -1226,7 +1307,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>79112790224</v>
       </c>
@@ -1237,7 +1318,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>79214489786</v>
       </c>
@@ -1248,7 +1329,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>79650289473</v>
       </c>
@@ -1259,7 +1340,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>79216581136</v>
       </c>
@@ -1270,7 +1351,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>79955992128</v>
       </c>
@@ -1281,7 +1362,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>79957502458</v>
       </c>
@@ -1292,7 +1373,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>79811319218</v>
       </c>
@@ -1303,7 +1384,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>79657607975</v>
       </c>
@@ -1314,7 +1395,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>79216439845</v>
       </c>
@@ -1325,7 +1406,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>79644151845</v>
       </c>
@@ -1336,7 +1417,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>79992100398</v>
       </c>
@@ -1347,7 +1428,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>79110209759</v>
       </c>
@@ -1358,7 +1439,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>79643752751</v>
       </c>
@@ -1369,7 +1450,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>79998764512</v>
       </c>
@@ -1380,7 +1461,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>79818406645</v>
       </c>
@@ -1391,7 +1472,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>77777777999</v>
       </c>
@@ -1402,7 +1483,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>79675539486</v>
       </c>
@@ -1413,7 +1494,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>79990050445</v>
       </c>
@@ -1424,7 +1505,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>79280562741</v>
       </c>
@@ -1435,7 +1516,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>79291543973</v>
       </c>
@@ -1446,7 +1527,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>79992154399</v>
       </c>
@@ -1457,7 +1538,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>79992348535</v>
       </c>
@@ -1468,7 +1549,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>79995312421</v>
       </c>
@@ -1479,7 +1560,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>79312394943</v>
       </c>
@@ -1490,7 +1571,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>79995369796</v>
       </c>
@@ -1501,7 +1582,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>79533799123</v>
       </c>
@@ -1512,7 +1593,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>79213578709</v>
       </c>
@@ -1523,7 +1604,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>79312394943</v>
       </c>
@@ -1534,7 +1615,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>79052128995</v>
       </c>
@@ -1545,7 +1626,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>79030963016</v>
       </c>
@@ -1556,7 +1637,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>79626897374</v>
       </c>
@@ -1567,7 +1648,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>79964989683</v>
       </c>
@@ -1578,7 +1659,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>79817394323</v>
       </c>
@@ -1589,7 +1670,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>79888782855</v>
       </c>
@@ -1600,9 +1681,9 @@
         <v>168</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45">
-        <v>79650767067</v>
+        <v>79632462321</v>
       </c>
       <c r="B45" t="s">
         <v>46</v>
@@ -1611,7 +1692,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>79112956224</v>
       </c>
@@ -1622,7 +1703,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>79812177760</v>
       </c>
@@ -1633,7 +1714,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>79930704547</v>
       </c>
@@ -1644,7 +1725,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>79522028041</v>
       </c>
@@ -1655,7 +1736,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>79618035054</v>
       </c>
@@ -1666,7 +1747,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>78889995511</v>
       </c>
@@ -1677,7 +1758,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>79995487895</v>
       </c>
@@ -1688,7 +1769,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>79616804670</v>
       </c>
@@ -1699,7 +1780,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>79300037229</v>
       </c>
@@ -1710,7 +1791,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>79998732422</v>
       </c>
@@ -1721,7 +1802,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>79997578106</v>
       </c>
@@ -1732,7 +1813,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>79114366261</v>
       </c>
@@ -1743,7 +1824,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>79602409094</v>
       </c>
@@ -1754,7 +1835,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>79995551199</v>
       </c>
@@ -1765,7 +1846,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>79998732488</v>
       </c>
@@ -1776,7 +1857,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>79668666673</v>
       </c>
@@ -1787,7 +1868,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>79213592462</v>
       </c>
@@ -1798,7 +1879,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>79992118912</v>
       </c>
@@ -1809,7 +1890,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>79696040964</v>
       </c>
@@ -1820,7 +1901,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>79602552759</v>
       </c>
@@ -1831,7 +1912,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>79992001264</v>
       </c>
@@ -1842,7 +1923,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>79045881207</v>
       </c>
@@ -1853,7 +1934,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>79788307253</v>
       </c>
@@ -1864,7 +1945,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>79523624780</v>
       </c>
@@ -1875,7 +1956,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>79522874320</v>
       </c>
@@ -1886,7 +1967,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>79117289353</v>
       </c>
@@ -1897,7 +1978,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>79944344427</v>
       </c>
@@ -1908,7 +1989,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>78887776655</v>
       </c>
@@ -1919,7 +2000,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>79216565223</v>
       </c>
@@ -1930,7 +2011,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>79817972145</v>
       </c>
@@ -1941,7 +2022,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="B76" t="s">
         <v>76</v>
       </c>
@@ -1949,7 +2030,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>79531483317</v>
       </c>
@@ -1960,7 +2041,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>79632429542</v>
       </c>
@@ -1971,7 +2052,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>79531661400</v>
       </c>
@@ -1982,7 +2063,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>79117032043</v>
       </c>
@@ -1993,7 +2074,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>79315825332</v>
       </c>
@@ -2004,7 +2085,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>79998068049</v>
       </c>
@@ -2015,7 +2096,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>79052532325</v>
       </c>
@@ -2026,7 +2107,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>79640707773</v>
       </c>
@@ -2037,7 +2118,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>79999998877</v>
       </c>
@@ -2048,7 +2129,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>79119970547</v>
       </c>
@@ -2059,7 +2140,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>79819664876</v>
       </c>
@@ -2070,7 +2151,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>79999998877</v>
       </c>
@@ -2081,7 +2162,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>79285372342</v>
       </c>
@@ -2092,7 +2173,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>79586760500</v>
       </c>
@@ -2103,7 +2184,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>79531709569</v>
       </c>
@@ -2114,7 +2195,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>79280969669</v>
       </c>
@@ -2125,7 +2206,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>79851512033</v>
       </c>
@@ -2136,7 +2217,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>79052632221</v>
       </c>
@@ -2147,7 +2228,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>79921744817</v>
       </c>
@@ -2158,7 +2239,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>79919909820</v>
       </c>
@@ -2169,7 +2250,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>79522015084</v>
       </c>
@@ -2180,7 +2261,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>70009998877</v>
       </c>
@@ -2191,7 +2272,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>79992080090</v>
       </c>
@@ -2202,7 +2283,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>79602818789</v>
       </c>
@@ -2213,7 +2294,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>79895461232</v>
       </c>
@@ -2224,7 +2305,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>79895461299</v>
       </c>
@@ -2235,7 +2316,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>79817264547</v>
       </c>
@@ -2246,7 +2327,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>79006450423</v>
       </c>
@@ -2257,7 +2338,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>79996753419</v>
       </c>
@@ -2268,7 +2349,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>79111780559</v>
       </c>
@@ -2279,7 +2360,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>79819673976</v>
       </c>
@@ -2290,7 +2371,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>79533777930</v>
       </c>
@@ -2301,7 +2382,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>79218681235</v>
       </c>
@@ -2312,7 +2393,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>79013797198</v>
       </c>
@@ -2323,7 +2404,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>79812686943</v>
       </c>
@@ -2334,7 +2415,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>79531644130</v>
       </c>
@@ -2345,7 +2426,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>79215678968</v>
       </c>
@@ -2356,7 +2437,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>79885673412</v>
       </c>
@@ -2367,7 +2448,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>799992357618</v>
       </c>
@@ -2378,7 +2459,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>79117221004</v>
       </c>
@@ -2389,7 +2470,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>79097589337</v>
       </c>
@@ -2400,7 +2481,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>79243944088</v>
       </c>
@@ -2411,7 +2492,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>79967944014</v>
       </c>
@@ -2422,7 +2503,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>79516734624</v>
       </c>
@@ -2433,7 +2514,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>79919965310</v>
       </c>
@@ -2444,7 +2525,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>79998741231</v>
       </c>
@@ -2455,7 +2536,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>79939708960</v>
       </c>
@@ -2466,7 +2547,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>79883256189</v>
       </c>
@@ -2477,7 +2558,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>79998881111</v>
       </c>
@@ -2488,18 +2569,32 @@
         <v>249</v>
       </c>
     </row>
+    <row r="126" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A126">
+        <v>79111326378</v>
+      </c>
+      <c r="B126" t="s">
+        <v>251</v>
+      </c>
+      <c r="C126" t="s">
+        <v>252</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="8.33203125" customWidth="1"/>
-    <col min="3" max="3" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="8.28515625" customWidth="1"/>
+    <col min="3" max="3" width="8.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2507,9 +2602,9 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>